<commit_message>
aggiunta SSD LanciaDadi, SpostaPedina, PassaDalVia
</commit_message>
<xml_diff>
--- a/Diagramma di Gantt.xlsx
+++ b/Diagramma di Gantt.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{948CD877-4746-4539-B5E8-3417178A8906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A45A4D9E-2BA8-4A79-B3AF-5DFA82A43CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1168,6 +1168,9 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="27" fillId="10" borderId="2" xfId="10" applyFont="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="8">
       <alignment horizontal="right" indent="1"/>
     </xf>
@@ -1186,64 +1189,61 @@
     <xf numFmtId="167" fontId="7" fillId="0" borderId="3" xfId="9">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="27" fillId="10" borderId="2" xfId="10" applyFont="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="54">
-    <cellStyle name="20% - Colore 1" xfId="31" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Colore 2" xfId="35" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Colore 3" xfId="39" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Colore 4" xfId="43" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Colore 5" xfId="47" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Colore 6" xfId="51" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Colore 1" xfId="32" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Colore 2" xfId="36" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Colore 3" xfId="40" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Colore 4" xfId="44" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Colore 5" xfId="48" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Colore 6" xfId="52" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Colore 1" xfId="33" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Colore 2" xfId="37" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Colore 3" xfId="41" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Colore 4" xfId="45" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Colore 5" xfId="49" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Colore 6" xfId="53" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="31" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="35" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="39" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="43" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="47" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="51" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="32" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="36" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="40" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="44" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="48" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="52" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="33" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="37" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="41" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="45" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="49" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="53" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="30" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="34" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="38" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="42" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="46" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="50" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Attività" xfId="12" xr:uid="{6391D789-272B-4DD2-9BF3-2CDCF610FA41}"/>
-    <cellStyle name="Calcolo" xfId="23" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Cella collegata" xfId="24" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Cella da controllare" xfId="25" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8" customBuiltin="1"/>
-    <cellStyle name="Collegamento ipertestuale visitato" xfId="13" builtinId="9" customBuiltin="1"/>
-    <cellStyle name="Colore 1" xfId="30" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Colore 2" xfId="34" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Colore 3" xfId="38" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Colore 4" xfId="42" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Colore 5" xfId="46" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Colore 6" xfId="50" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="19" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="23" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="25" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Comma" xfId="4" builtinId="3" customBuiltin="1"/>
+    <cellStyle name="Comma [0]" xfId="14" builtinId="6" customBuiltin="1"/>
+    <cellStyle name="Currency" xfId="15" builtinId="4" customBuiltin="1"/>
+    <cellStyle name="Currency [0]" xfId="16" builtinId="7" customBuiltin="1"/>
     <cellStyle name="Data" xfId="10" xr:uid="{229918B6-DD13-4F5A-97B9-305F7E002AA3}"/>
+    <cellStyle name="Explanatory Text" xfId="28" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="13" builtinId="9" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="18" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="6" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="7" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="8" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="17" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" customBuiltin="1"/>
     <cellStyle name="Inizio progetto" xfId="9" xr:uid="{8EB8A09A-C31C-40A3-B2C1-9449520178B8}"/>
     <cellStyle name="Input" xfId="21" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Migliaia" xfId="4" builtinId="3" customBuiltin="1"/>
-    <cellStyle name="Migliaia [0]" xfId="14" builtinId="6" customBuiltin="1"/>
-    <cellStyle name="Neutrale" xfId="20" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="24" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="20" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Nome" xfId="11" xr:uid="{B2D3C1EE-6B41-4801-AAFC-C2274E49E503}"/>
-    <cellStyle name="Normale" xfId="0" builtinId="0" customBuiltin="1"/>
-    <cellStyle name="Nota" xfId="27" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="27" builtinId="10" customBuiltin="1"/>
     <cellStyle name="Output" xfId="22" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Percentuale" xfId="2" builtinId="5" customBuiltin="1"/>
-    <cellStyle name="Testo avviso" xfId="26" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Testo descrittivo" xfId="28" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Titolo" xfId="5" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Titolo 1" xfId="6" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Titolo 2" xfId="7" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Titolo 3" xfId="8" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Titolo 4" xfId="17" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Totale" xfId="29" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Valore non valido" xfId="19" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Valore valido" xfId="18" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Valuta" xfId="15" builtinId="4" customBuiltin="1"/>
-    <cellStyle name="Valuta [0]" xfId="16" builtinId="7" customBuiltin="1"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="5" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="29" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="26" builtinId="11" customBuiltin="1"/>
     <cellStyle name="zTestoNascosto" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
   <dxfs count="14">
@@ -1807,97 +1807,97 @@
       <c r="B3" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="73" t="s">
+      <c r="C3" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="74"/>
-      <c r="E3" s="78">
+      <c r="D3" s="75"/>
+      <c r="E3" s="79">
         <f ca="1">TODAY()</f>
-        <v>45649</v>
-      </c>
-      <c r="F3" s="78"/>
+        <v>45650</v>
+      </c>
+      <c r="F3" s="79"/>
     </row>
     <row r="4" spans="1:56" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="73" t="s">
+      <c r="C4" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="74"/>
+      <c r="D4" s="75"/>
       <c r="E4" s="6">
         <v>1</v>
       </c>
-      <c r="H4" s="75">
+      <c r="H4" s="76">
         <f ca="1">H5</f>
         <v>45649</v>
       </c>
-      <c r="I4" s="76"/>
-      <c r="J4" s="76"/>
-      <c r="K4" s="76"/>
-      <c r="L4" s="76"/>
-      <c r="M4" s="76"/>
-      <c r="N4" s="77"/>
-      <c r="O4" s="75">
+      <c r="I4" s="77"/>
+      <c r="J4" s="77"/>
+      <c r="K4" s="77"/>
+      <c r="L4" s="77"/>
+      <c r="M4" s="77"/>
+      <c r="N4" s="78"/>
+      <c r="O4" s="76">
         <f ca="1">O5</f>
         <v>45656</v>
       </c>
-      <c r="P4" s="76"/>
-      <c r="Q4" s="76"/>
-      <c r="R4" s="76"/>
-      <c r="S4" s="76"/>
-      <c r="T4" s="76"/>
-      <c r="U4" s="77"/>
-      <c r="V4" s="75">
+      <c r="P4" s="77"/>
+      <c r="Q4" s="77"/>
+      <c r="R4" s="77"/>
+      <c r="S4" s="77"/>
+      <c r="T4" s="77"/>
+      <c r="U4" s="78"/>
+      <c r="V4" s="76">
         <f ca="1">V5</f>
         <v>45663</v>
       </c>
-      <c r="W4" s="76"/>
-      <c r="X4" s="76"/>
-      <c r="Y4" s="76"/>
-      <c r="Z4" s="76"/>
-      <c r="AA4" s="76"/>
-      <c r="AB4" s="77"/>
-      <c r="AC4" s="75">
+      <c r="W4" s="77"/>
+      <c r="X4" s="77"/>
+      <c r="Y4" s="77"/>
+      <c r="Z4" s="77"/>
+      <c r="AA4" s="77"/>
+      <c r="AB4" s="78"/>
+      <c r="AC4" s="76">
         <f ca="1">AC5</f>
         <v>45670</v>
       </c>
-      <c r="AD4" s="76"/>
-      <c r="AE4" s="76"/>
-      <c r="AF4" s="76"/>
-      <c r="AG4" s="76"/>
-      <c r="AH4" s="76"/>
-      <c r="AI4" s="77"/>
-      <c r="AJ4" s="75">
+      <c r="AD4" s="77"/>
+      <c r="AE4" s="77"/>
+      <c r="AF4" s="77"/>
+      <c r="AG4" s="77"/>
+      <c r="AH4" s="77"/>
+      <c r="AI4" s="78"/>
+      <c r="AJ4" s="76">
         <f ca="1">AJ5</f>
         <v>45677</v>
       </c>
-      <c r="AK4" s="76"/>
-      <c r="AL4" s="76"/>
-      <c r="AM4" s="76"/>
-      <c r="AN4" s="76"/>
-      <c r="AO4" s="76"/>
-      <c r="AP4" s="77"/>
-      <c r="AQ4" s="75">
+      <c r="AK4" s="77"/>
+      <c r="AL4" s="77"/>
+      <c r="AM4" s="77"/>
+      <c r="AN4" s="77"/>
+      <c r="AO4" s="77"/>
+      <c r="AP4" s="78"/>
+      <c r="AQ4" s="76">
         <f ca="1">AQ5</f>
         <v>45684</v>
       </c>
-      <c r="AR4" s="76"/>
-      <c r="AS4" s="76"/>
-      <c r="AT4" s="76"/>
-      <c r="AU4" s="76"/>
-      <c r="AV4" s="76"/>
-      <c r="AW4" s="77"/>
-      <c r="AX4" s="75">
+      <c r="AR4" s="77"/>
+      <c r="AS4" s="77"/>
+      <c r="AT4" s="77"/>
+      <c r="AU4" s="77"/>
+      <c r="AV4" s="77"/>
+      <c r="AW4" s="78"/>
+      <c r="AX4" s="76">
         <f ca="1">AX5</f>
         <v>45691</v>
       </c>
-      <c r="AY4" s="76"/>
-      <c r="AZ4" s="76"/>
-      <c r="BA4" s="76"/>
-      <c r="BB4" s="76"/>
-      <c r="BC4" s="76"/>
-      <c r="BD4" s="77"/>
+      <c r="AY4" s="77"/>
+      <c r="AZ4" s="77"/>
+      <c r="BA4" s="77"/>
+      <c r="BB4" s="77"/>
+      <c r="BC4" s="77"/>
+      <c r="BD4" s="78"/>
     </row>
     <row r="5" spans="1:56" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
@@ -2458,15 +2458,15 @@
         <v>43</v>
       </c>
       <c r="D9" s="13">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E9" s="48">
         <f ca="1">Inizio_progetto</f>
-        <v>45649</v>
+        <v>45650</v>
       </c>
       <c r="F9" s="48">
         <f ca="1">E9</f>
-        <v>45649</v>
+        <v>45650</v>
       </c>
       <c r="G9" s="10">
         <f t="shared" ref="G9:G26" ca="1" si="5">IF(OR(ISBLANK(inizio_attività),ISBLANK(fine_attività)),"",fine_attività-inizio_attività+1)</f>
@@ -2531,15 +2531,15 @@
         <v>35</v>
       </c>
       <c r="D10" s="13">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="E10" s="48">
         <f ca="1">F9</f>
-        <v>45649</v>
+        <v>45650</v>
       </c>
       <c r="F10" s="48">
         <f ca="1">E10</f>
-        <v>45649</v>
+        <v>45650</v>
       </c>
       <c r="G10" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -2667,15 +2667,15 @@
         <v>36</v>
       </c>
       <c r="D12" s="16">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="E12" s="51">
         <f ca="1">F10</f>
-        <v>45649</v>
+        <v>45650</v>
       </c>
       <c r="F12" s="51">
         <f ca="1">E12</f>
-        <v>45649</v>
+        <v>45650</v>
       </c>
       <c r="G12" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -2740,15 +2740,15 @@
         <v>43</v>
       </c>
       <c r="D13" s="16">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="E13" s="51">
         <f ca="1">E12+1</f>
-        <v>45650</v>
+        <v>45651</v>
       </c>
       <c r="F13" s="51">
         <f t="shared" ref="F13:F15" ca="1" si="6">E13</f>
-        <v>45650</v>
+        <v>45651</v>
       </c>
       <c r="G13" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -2813,15 +2813,15 @@
         <v>43</v>
       </c>
       <c r="D14" s="16">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="E14" s="51">
         <f ca="1">E13</f>
-        <v>45650</v>
+        <v>45651</v>
       </c>
       <c r="F14" s="51">
         <f t="shared" ca="1" si="6"/>
-        <v>45650</v>
+        <v>45651</v>
       </c>
       <c r="G14" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -2890,11 +2890,11 @@
       </c>
       <c r="E15" s="51">
         <f t="shared" ref="E15" ca="1" si="7">E14</f>
-        <v>45650</v>
+        <v>45651</v>
       </c>
       <c r="F15" s="51">
         <f t="shared" ca="1" si="6"/>
-        <v>45650</v>
+        <v>45651</v>
       </c>
       <c r="G15" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -2963,11 +2963,11 @@
       </c>
       <c r="E16" s="51">
         <f ca="1">F15+2</f>
-        <v>45652</v>
+        <v>45653</v>
       </c>
       <c r="F16" s="51">
         <f ca="1">E16</f>
-        <v>45652</v>
+        <v>45653</v>
       </c>
       <c r="G16" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3036,11 +3036,11 @@
       </c>
       <c r="E17" s="51">
         <f ca="1">E16</f>
-        <v>45652</v>
+        <v>45653</v>
       </c>
       <c r="F17" s="51">
         <f ca="1">E17</f>
-        <v>45652</v>
+        <v>45653</v>
       </c>
       <c r="G17" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3109,11 +3109,11 @@
       </c>
       <c r="E18" s="51">
         <f ca="1">E17</f>
-        <v>45652</v>
+        <v>45653</v>
       </c>
       <c r="F18" s="51">
         <f ca="1">E18</f>
-        <v>45652</v>
+        <v>45653</v>
       </c>
       <c r="G18" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3182,11 +3182,11 @@
       </c>
       <c r="E19" s="51">
         <f ca="1">E13</f>
-        <v>45650</v>
+        <v>45651</v>
       </c>
       <c r="F19" s="51">
         <f ca="1">E19+2</f>
-        <v>45652</v>
+        <v>45653</v>
       </c>
       <c r="G19" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3255,11 +3255,11 @@
       </c>
       <c r="E20" s="51">
         <f ca="1">F19+1</f>
-        <v>45653</v>
+        <v>45654</v>
       </c>
       <c r="F20" s="51">
         <f ca="1">E20+1</f>
-        <v>45654</v>
+        <v>45655</v>
       </c>
       <c r="G20" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3391,11 +3391,11 @@
       </c>
       <c r="E22" s="54">
         <f ca="1">F20+1</f>
-        <v>45655</v>
+        <v>45656</v>
       </c>
       <c r="F22" s="54">
         <f ca="1">E22+7</f>
-        <v>45662</v>
+        <v>45663</v>
       </c>
       <c r="G22" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3464,11 +3464,11 @@
       </c>
       <c r="E23" s="54">
         <f ca="1">E22</f>
-        <v>45655</v>
+        <v>45656</v>
       </c>
       <c r="F23" s="54">
         <f ca="1">E23+7</f>
-        <v>45662</v>
+        <v>45663</v>
       </c>
       <c r="G23" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3537,11 +3537,11 @@
       </c>
       <c r="E24" s="54">
         <f ca="1">E23</f>
-        <v>45655</v>
+        <v>45656</v>
       </c>
       <c r="F24" s="54">
         <f ca="1">E24+3</f>
-        <v>45658</v>
+        <v>45659</v>
       </c>
       <c r="G24" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3610,11 +3610,11 @@
       </c>
       <c r="E25" s="54">
         <f ca="1">F22+1</f>
-        <v>45663</v>
+        <v>45664</v>
       </c>
       <c r="F25" s="54">
         <f ca="1">E25+4</f>
-        <v>45667</v>
+        <v>45668</v>
       </c>
       <c r="G25" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3683,11 +3683,11 @@
       </c>
       <c r="E26" s="54">
         <f ca="1">F25-1</f>
-        <v>45666</v>
-      </c>
-      <c r="F26" s="79">
+        <v>45667</v>
+      </c>
+      <c r="F26" s="73">
         <f ca="1">E26+2</f>
-        <v>45668</v>
+        <v>45669</v>
       </c>
       <c r="G26" s="10">
         <f t="shared" ca="1" si="5"/>
@@ -3819,11 +3819,11 @@
       </c>
       <c r="E28" s="57">
         <f ca="1">F25+1</f>
-        <v>45668</v>
+        <v>45669</v>
       </c>
       <c r="F28" s="57">
         <f ca="1">E28+3</f>
-        <v>45671</v>
+        <v>45672</v>
       </c>
       <c r="G28" s="10">
         <f t="shared" ca="1" si="8"/>
@@ -3957,11 +3957,11 @@
       </c>
       <c r="E30" s="54">
         <f ca="1">F28</f>
-        <v>45671</v>
+        <v>45672</v>
       </c>
       <c r="F30" s="54">
         <f ca="1">E30+5</f>
-        <v>45676</v>
+        <v>45677</v>
       </c>
       <c r="G30" s="10">
         <f t="shared" ca="1" si="8"/>
@@ -4030,11 +4030,11 @@
       </c>
       <c r="E31" s="54">
         <f ca="1">E30</f>
-        <v>45671</v>
+        <v>45672</v>
       </c>
       <c r="F31" s="54">
         <f ca="1">E31+5</f>
-        <v>45676</v>
+        <v>45677</v>
       </c>
       <c r="G31" s="10">
         <f t="shared" ca="1" si="8"/>
@@ -4103,11 +4103,11 @@
       </c>
       <c r="E32" s="54">
         <f ca="1">E31</f>
-        <v>45671</v>
+        <v>45672</v>
       </c>
       <c r="F32" s="54">
         <f ca="1">E32+3</f>
-        <v>45674</v>
+        <v>45675</v>
       </c>
       <c r="G32" s="10">
         <f t="shared" ca="1" si="8"/>
@@ -4176,11 +4176,11 @@
       </c>
       <c r="E33" s="54">
         <f ca="1">F30+1</f>
-        <v>45677</v>
+        <v>45678</v>
       </c>
       <c r="F33" s="54">
         <f ca="1">E33+2</f>
-        <v>45679</v>
+        <v>45680</v>
       </c>
       <c r="G33" s="10">
         <f t="shared" ca="1" si="8"/>
@@ -4249,11 +4249,11 @@
       </c>
       <c r="E34" s="54">
         <f ca="1">F33-1</f>
-        <v>45678</v>
+        <v>45679</v>
       </c>
       <c r="F34" s="54">
         <f ca="1">E34+1</f>
-        <v>45679</v>
+        <v>45680</v>
       </c>
       <c r="G34" s="10">
         <f t="shared" ca="1" si="8"/>
@@ -4382,11 +4382,11 @@
       </c>
       <c r="E36" s="57">
         <f ca="1">F34+1</f>
-        <v>45680</v>
+        <v>45681</v>
       </c>
       <c r="F36" s="57">
         <f ca="1">E36+3</f>
-        <v>45683</v>
+        <v>45684</v>
       </c>
       <c r="G36" s="10">
         <f ca="1">IF(OR(ISBLANK(inizio_attività),ISBLANK(fine_attività)),"",fine_attività-inizio_attività+1)</f>
@@ -4455,11 +4455,11 @@
       </c>
       <c r="E37" s="57">
         <f ca="1">F36</f>
-        <v>45683</v>
+        <v>45684</v>
       </c>
       <c r="F37" s="57">
         <f ca="1">F36</f>
-        <v>45683</v>
+        <v>45684</v>
       </c>
       <c r="G37" s="10">
         <f ca="1">IF(OR(ISBLANK(inizio_attività),ISBLANK(fine_attività)),"",fine_attività-inizio_attività+1)</f>
@@ -4625,6 +4625,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101003574973502B84C42B74035BA8AADE1A3" ma:contentTypeVersion="9" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="1ba771f4a91505810405fb99ac35d176">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8f4f0557-6568-4af7-94c6-f11cb446b9b2" xmlns:ns4="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3481e8909782aae8d117dfcc8e1ba87" ns3:_="" ns4:_="">
     <xsd:import namespace="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
@@ -4819,24 +4836,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A7A2A5-3EAC-4111-8CE5-4F4CD491981F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4853,29 +4878,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modifica AD e gantt
</commit_message>
<xml_diff>
--- a/Diagramma di Gantt.xlsx
+++ b/Diagramma di Gantt.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B98E4B0-6ECD-4569-A369-5CAE2C233606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A947D93-FB68-46C1-B930-C26BDEAFC42E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PianificazioneProgetto" sheetId="11" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">
   <si>
     <t>Come creare la pianificazione di un progetto in questo foglio di lavoro.
 Immettere il titolo del progetto nella cella B1. 
@@ -174,9 +174,6 @@
   </si>
   <si>
     <t>Implementazione del database</t>
-  </si>
-  <si>
-    <t>Teruzzi, Messa</t>
   </si>
   <si>
     <t>Tentori, Ronchi</t>
@@ -226,7 +223,7 @@
     <numFmt numFmtId="168" formatCode="d\ mmm\ yyyy"/>
     <numFmt numFmtId="169" formatCode="d"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,6 +414,13 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -959,7 +963,7 @@
     <xf numFmtId="0" fontId="7" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1176,6 +1180,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="3" xfId="9">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="27" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1771,7 +1778,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
@@ -1785,7 +1792,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H2" s="45"/>
     </row>
@@ -2095,7 +2102,7 @@
     </row>
     <row r="6" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="69" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>6</v>
@@ -2443,7 +2450,7 @@
         <v>15</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D9" s="13">
         <v>1</v>
@@ -2725,7 +2732,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D13" s="16">
         <v>0.9</v>
@@ -2798,7 +2805,7 @@
         <v>24</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D14" s="16">
         <v>0.4</v>
@@ -2871,7 +2878,7 @@
         <v>25</v>
       </c>
       <c r="C15" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D15" s="16">
         <v>0.4</v>
@@ -2944,10 +2951,10 @@
         <v>26</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16" s="16">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E16" s="51">
         <f>F13+1</f>
@@ -3017,10 +3024,10 @@
         <v>27</v>
       </c>
       <c r="C17" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D17" s="16">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E17" s="51">
         <f>E16</f>
@@ -3090,7 +3097,7 @@
         <v>28</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D18" s="16">
         <v>0.8</v>
@@ -3163,7 +3170,7 @@
         <v>17</v>
       </c>
       <c r="C19" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D19" s="16">
         <v>0</v>
@@ -3236,10 +3243,10 @@
         <v>40</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="D20" s="16">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="E20" s="51">
         <f>E19</f>
@@ -3309,7 +3316,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="35"/>
-      <c r="D21" s="18"/>
+      <c r="D21" s="78"/>
       <c r="E21" s="52"/>
       <c r="F21" s="53"/>
       <c r="G21" s="10" t="str">
@@ -3369,10 +3376,10 @@
     <row r="22" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="67"/>
       <c r="B22" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="36" t="s">
         <v>44</v>
-      </c>
-      <c r="C22" s="36" t="s">
-        <v>45</v>
       </c>
       <c r="D22" s="19">
         <v>0</v>
@@ -3733,7 +3740,7 @@
     <row r="27" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="20"/>
       <c r="B27" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C27" s="37"/>
       <c r="D27" s="21"/>
@@ -3796,7 +3803,7 @@
     <row r="28" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="42"/>
       <c r="B28" s="42" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C28" s="38" t="s">
         <v>33</v>
@@ -3934,10 +3941,10 @@
     <row r="30" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="41"/>
       <c r="B30" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" s="36" t="s">
         <v>44</v>
-      </c>
-      <c r="C30" s="36" t="s">
-        <v>45</v>
       </c>
       <c r="D30" s="19">
         <v>0</v>
@@ -4299,7 +4306,7 @@
     <row r="35" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="20"/>
       <c r="B35" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C35" s="37"/>
       <c r="D35" s="21"/>
@@ -4359,7 +4366,7 @@
     <row r="36" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="42"/>
       <c r="B36" s="42" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C36" s="38" t="s">
         <v>33</v>
@@ -4612,23 +4619,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101003574973502B84C42B74035BA8AADE1A3" ma:contentTypeVersion="9" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="1ba771f4a91505810405fb99ac35d176">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8f4f0557-6568-4af7-94c6-f11cb446b9b2" xmlns:ns4="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3481e8909782aae8d117dfcc8e1ba87" ns3:_="" ns4:_="">
     <xsd:import namespace="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
@@ -4823,32 +4813,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A7A2A5-3EAC-4111-8CE5-4F4CD491981F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4865,4 +4847,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Aggiornamento diagramma di Gantt
</commit_message>
<xml_diff>
--- a/Diagramma di Gantt.xlsx
+++ b/Diagramma di Gantt.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C963F21E-0EFB-4A86-B687-3E514412D4A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A312E701-743B-415A-83C6-AC4B690795F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="62">
   <si>
     <t>Come creare la pianificazione di un progetto in questo foglio di lavoro.
 Immettere il titolo del progetto nella cella B1. 
@@ -149,12 +149,6 @@
     <t>Tentori</t>
   </si>
   <si>
-    <t>Ronchi, Messa</t>
-  </si>
-  <si>
-    <t>Tentori, Teruzzi</t>
-  </si>
-  <si>
     <t>Messa</t>
   </si>
   <si>
@@ -182,9 +176,6 @@
     <t xml:space="preserve">Sviluppo del backend </t>
   </si>
   <si>
-    <t>Messa, Ronchi</t>
-  </si>
-  <si>
     <t>ITERAZIONE</t>
   </si>
   <si>
@@ -213,6 +204,36 @@
   </si>
   <si>
     <t>Ricerca React</t>
+  </si>
+  <si>
+    <t>Teruzzi, Messa</t>
+  </si>
+  <si>
+    <t>Tentori, Ronchi, Messa</t>
+  </si>
+  <si>
+    <t>Ronchi, Messa, Tentori</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Revisione diagrammi</t>
+  </si>
+  <si>
+    <t>Teruzzi, Messa, Ronchi</t>
+  </si>
+  <si>
+    <t>Revisione del database</t>
+  </si>
+  <si>
+    <t>Ronchi, Tentori</t>
+  </si>
+  <si>
+    <t>Ronchi, Messa, Tentori, Teruzzi</t>
+  </si>
+  <si>
+    <t>Tentori, Teruzzi, Ronchi, Messa</t>
   </si>
 </sst>
 </file>
@@ -969,7 +990,7 @@
     <xf numFmtId="0" fontId="7" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1189,6 +1210,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="3" xfId="9">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1765,7 +1789,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BD39"/>
+  <dimension ref="A1:BD40"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" style="25" customWidth="1"/>
@@ -1784,7 +1808,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="28" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
@@ -1798,7 +1822,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="29" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="H2" s="45"/>
     </row>
@@ -1807,7 +1831,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C3" s="73" t="s">
         <v>7</v>
@@ -2108,7 +2132,7 @@
     </row>
     <row r="6" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="69" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>6</v>
@@ -2456,7 +2480,7 @@
         <v>15</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D9" s="13">
         <v>1</v>
@@ -2529,10 +2553,10 @@
         <v>21</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D10" s="13">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E10" s="48">
         <f>F9</f>
@@ -2665,10 +2689,10 @@
         <v>22</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D12" s="16">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E12" s="51">
         <f>F10+1</f>
@@ -2738,10 +2762,10 @@
         <v>23</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D13" s="16">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E13" s="51">
         <f>E12</f>
@@ -2811,10 +2835,10 @@
         <v>24</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D14" s="16">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E14" s="51">
         <f>E13</f>
@@ -2884,10 +2908,10 @@
         <v>25</v>
       </c>
       <c r="C15" s="34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D15" s="16">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E15" s="51">
         <f>E14</f>
@@ -2957,10 +2981,10 @@
         <v>26</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D16" s="16">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E16" s="51">
         <f>F13+1</f>
@@ -3030,10 +3054,10 @@
         <v>27</v>
       </c>
       <c r="C17" s="34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D17" s="16">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E17" s="51">
         <f>E16</f>
@@ -3103,10 +3127,10 @@
         <v>28</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D18" s="16">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E18" s="51">
         <f>E17</f>
@@ -3176,10 +3200,10 @@
         <v>17</v>
       </c>
       <c r="C19" s="34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D19" s="16">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E19" s="51">
         <f>F18</f>
@@ -3246,16 +3270,16 @@
     <row r="20" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="40"/>
       <c r="B20" s="40" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C20" s="34" t="s">
         <v>31</v>
       </c>
       <c r="D20" s="16">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="E20" s="51">
-        <f t="shared" ref="E20:E21" si="6">F19</f>
+        <f t="shared" ref="E20" si="6">F19</f>
         <v>45660</v>
       </c>
       <c r="F20" s="51">
@@ -3316,13 +3340,13 @@
     <row r="21" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="40"/>
       <c r="B21" s="40" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C21" s="34" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D21" s="16">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="51">
         <f>E20</f>
@@ -3386,25 +3410,25 @@
     <row r="22" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="40"/>
       <c r="B22" s="40" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C22" s="34" t="s">
         <v>32</v>
       </c>
       <c r="D22" s="16">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E22" s="51">
         <f>E19</f>
         <v>45660</v>
       </c>
       <c r="F22" s="51">
-        <f>E22</f>
-        <v>45660</v>
+        <f>E22+1</f>
+        <v>45661</v>
       </c>
       <c r="G22" s="10">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22" s="71"/>
       <c r="I22" s="71"/>
@@ -3522,24 +3546,24 @@
     <row r="24" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="67"/>
       <c r="B24" s="41" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D24" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="54">
         <v>45661</v>
       </c>
       <c r="F24" s="54">
-        <f>E24+5</f>
-        <v>45666</v>
+        <f>E24+17</f>
+        <v>45678</v>
       </c>
       <c r="G24" s="10">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H24" s="71"/>
       <c r="I24" s="71"/>
@@ -3597,22 +3621,22 @@
         <v>19</v>
       </c>
       <c r="C25" s="36" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D25" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" s="54">
         <f>E24</f>
         <v>45661</v>
       </c>
       <c r="F25" s="54">
-        <f>E25+5</f>
-        <v>45666</v>
+        <f>E25+17</f>
+        <v>45678</v>
       </c>
       <c r="G25" s="10">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H25" s="71"/>
       <c r="I25" s="71"/>
@@ -3667,25 +3691,25 @@
     <row r="26" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="67"/>
       <c r="B26" s="41" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C26" s="36" t="s">
         <v>32</v>
       </c>
       <c r="D26" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" s="54">
         <f>E25</f>
         <v>45661</v>
       </c>
       <c r="F26" s="54">
-        <f>E26+3</f>
-        <v>45664</v>
+        <f>E26+6</f>
+        <v>45667</v>
       </c>
       <c r="G26" s="10">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H26" s="71"/>
       <c r="I26" s="71"/>
@@ -3743,18 +3767,18 @@
         <v>30</v>
       </c>
       <c r="C27" s="36" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="D27" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="54">
-        <f>F24+1</f>
-        <v>45667</v>
+        <f>E24+17</f>
+        <v>45678</v>
       </c>
       <c r="F27" s="54">
         <f>E27+4</f>
-        <v>45671</v>
+        <v>45682</v>
       </c>
       <c r="G27" s="10">
         <f t="shared" si="5"/>
@@ -3816,22 +3840,22 @@
         <v>20</v>
       </c>
       <c r="C28" s="36" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D28" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" s="54">
-        <f>F27-1</f>
-        <v>45670</v>
+        <f>E27+1</f>
+        <v>45679</v>
       </c>
       <c r="F28" s="54">
-        <f>E28+2</f>
-        <v>45672</v>
+        <f>E28</f>
+        <v>45679</v>
       </c>
       <c r="G28" s="10">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H28" s="71"/>
       <c r="I28" s="71"/>
@@ -3886,14 +3910,14 @@
     <row r="29" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="20"/>
       <c r="B29" s="20" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C29" s="37"/>
       <c r="D29" s="21"/>
       <c r="E29" s="55"/>
       <c r="F29" s="56"/>
       <c r="G29" s="10" t="str">
-        <f t="shared" ref="G29:G36" si="7">IF(OR(ISBLANK(inizio_attività),ISBLANK(fine_attività)),"",fine_attività-inizio_attività+1)</f>
+        <f t="shared" ref="G29:G37" si="7">IF(OR(ISBLANK(inizio_attività),ISBLANK(fine_attività)),"",fine_attività-inizio_attività+1)</f>
         <v/>
       </c>
       <c r="H29" s="71"/>
@@ -3949,21 +3973,21 @@
     <row r="30" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="42"/>
       <c r="B30" s="42" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C30" s="38" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="D30" s="22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" s="57">
-        <f>F27+1</f>
-        <v>45672</v>
+        <f>F28</f>
+        <v>45679</v>
       </c>
       <c r="F30" s="57">
         <f>E30+3</f>
-        <v>45675</v>
+        <v>45682</v>
       </c>
       <c r="G30" s="10">
         <f t="shared" si="7"/>
@@ -4020,19 +4044,18 @@
       <c r="BD30" s="23"/>
     </row>
     <row r="31" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="66">
+      <c r="A31" s="79">
         <v>2</v>
       </c>
-      <c r="B31" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" s="35"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="52"/>
-      <c r="F31" s="53"/>
-      <c r="G31" s="10" t="str">
-        <f t="shared" si="7"/>
-        <v/>
+      <c r="B31" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="33"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="50"/>
+      <c r="G31" s="10" t="s">
+        <v>55</v>
       </c>
       <c r="H31" s="71"/>
       <c r="I31" s="71"/>
@@ -4085,27 +4108,26 @@
       <c r="BD31" s="23"/>
     </row>
     <row r="32" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="41"/>
-      <c r="B32" s="41" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" s="19">
-        <v>0</v>
-      </c>
-      <c r="E32" s="54">
+      <c r="A32" s="40"/>
+      <c r="B32" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="D32" s="16">
+        <v>1</v>
+      </c>
+      <c r="E32" s="51">
         <f>F30</f>
-        <v>45675</v>
-      </c>
-      <c r="F32" s="54">
-        <f>E32+5</f>
-        <v>45680</v>
+        <v>45682</v>
+      </c>
+      <c r="F32" s="51">
+        <f>E32+4</f>
+        <v>45686</v>
       </c>
       <c r="G32" s="10">
-        <f t="shared" si="7"/>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H32" s="71"/>
       <c r="I32" s="71"/>
@@ -4157,28 +4179,18 @@
       <c r="BC32" s="23"/>
       <c r="BD32" s="23"/>
     </row>
-    <row r="33" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="41"/>
-      <c r="B33" s="41" t="s">
-        <v>19</v>
-      </c>
-      <c r="C33" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="D33" s="19">
-        <v>0</v>
-      </c>
-      <c r="E33" s="54">
-        <f>E32</f>
-        <v>45675</v>
-      </c>
-      <c r="F33" s="54">
-        <f>E33+5</f>
-        <v>45680</v>
-      </c>
-      <c r="G33" s="10">
+    <row r="33" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="66"/>
+      <c r="B33" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="35"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="52"/>
+      <c r="F33" s="53"/>
+      <c r="G33" s="10" t="str">
         <f t="shared" si="7"/>
-        <v>6</v>
+        <v/>
       </c>
       <c r="H33" s="71"/>
       <c r="I33" s="71"/>
@@ -4230,28 +4242,28 @@
       <c r="BC33" s="23"/>
       <c r="BD33" s="23"/>
     </row>
-    <row r="34" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="41"/>
       <c r="B34" s="41" t="s">
         <v>41</v>
       </c>
       <c r="C34" s="36" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="D34" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" s="54">
-        <f>E33</f>
-        <v>45675</v>
+        <f>F30</f>
+        <v>45682</v>
       </c>
       <c r="F34" s="54">
-        <f>E34+3</f>
-        <v>45678</v>
+        <f>E34+2</f>
+        <v>45684</v>
       </c>
       <c r="G34" s="10">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H34" s="71"/>
       <c r="I34" s="71"/>
@@ -4306,21 +4318,21 @@
     <row r="35" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="41"/>
       <c r="B35" s="41" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="C35" s="36" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="D35" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" s="54">
-        <f>F32+1</f>
-        <v>45681</v>
+        <f>E34</f>
+        <v>45682</v>
       </c>
       <c r="F35" s="54">
         <f>E35+2</f>
-        <v>45683</v>
+        <v>45684</v>
       </c>
       <c r="G35" s="10">
         <f t="shared" si="7"/>
@@ -4377,27 +4389,27 @@
       <c r="BD35" s="23"/>
     </row>
     <row r="36" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="61"/>
-      <c r="B36" s="61" t="s">
-        <v>20</v>
+      <c r="A36" s="41"/>
+      <c r="B36" s="41" t="s">
+        <v>58</v>
       </c>
       <c r="C36" s="36" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D36" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="54">
-        <f>F35-1</f>
+        <f>E35</f>
         <v>45682</v>
       </c>
       <c r="F36" s="54">
-        <f>E36+1</f>
-        <v>45683</v>
+        <f>E36</f>
+        <v>45682</v>
       </c>
       <c r="G36" s="10">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" s="71"/>
       <c r="I36" s="71"/>
@@ -4450,15 +4462,28 @@
       <c r="BD36" s="23"/>
     </row>
     <row r="37" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="20"/>
-      <c r="B37" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="C37" s="37"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="56"/>
-      <c r="G37" s="10"/>
+      <c r="A37" s="41"/>
+      <c r="B37" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D37" s="19">
+        <v>1</v>
+      </c>
+      <c r="E37" s="54">
+        <f>F34</f>
+        <v>45684</v>
+      </c>
+      <c r="F37" s="54">
+        <f>E37+1</f>
+        <v>45685</v>
+      </c>
+      <c r="G37" s="10">
+        <f t="shared" si="7"/>
+        <v>2</v>
+      </c>
       <c r="H37" s="71"/>
       <c r="I37" s="71"/>
       <c r="J37" s="71"/>
@@ -4509,29 +4534,16 @@
       <c r="BC37" s="23"/>
       <c r="BD37" s="23"/>
     </row>
-    <row r="38" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="42"/>
-      <c r="B38" s="42" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38" s="38" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" s="22">
-        <v>0</v>
-      </c>
-      <c r="E38" s="57">
-        <f>F36+1</f>
-        <v>45684</v>
-      </c>
-      <c r="F38" s="57">
-        <f>E38+3</f>
-        <v>45687</v>
-      </c>
-      <c r="G38" s="10">
-        <f>IF(OR(ISBLANK(inizio_attività),ISBLANK(fine_attività)),"",fine_attività-inizio_attività+1)</f>
-        <v>4</v>
-      </c>
+    <row r="38" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="20"/>
+      <c r="B38" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="37"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="55"/>
+      <c r="F38" s="56"/>
+      <c r="G38" s="10"/>
       <c r="H38" s="71"/>
       <c r="I38" s="71"/>
       <c r="J38" s="71"/>
@@ -4582,28 +4594,28 @@
       <c r="BC38" s="23"/>
       <c r="BD38" s="23"/>
     </row>
-    <row r="39" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:56" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="42"/>
       <c r="B39" s="42" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C39" s="38" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="D39" s="22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" s="57">
-        <f>F38</f>
-        <v>45687</v>
+        <f>F35</f>
+        <v>45684</v>
       </c>
       <c r="F39" s="57">
-        <f>F38</f>
-        <v>45687</v>
+        <f>E39+2</f>
+        <v>45686</v>
       </c>
       <c r="G39" s="10">
         <f>IF(OR(ISBLANK(inizio_attività),ISBLANK(fine_attività)),"",fine_attività-inizio_attività+1)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H39" s="71"/>
       <c r="I39" s="71"/>
@@ -4655,6 +4667,79 @@
       <c r="BC39" s="23"/>
       <c r="BD39" s="23"/>
     </row>
+    <row r="40" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="42"/>
+      <c r="B40" s="42" t="s">
+        <v>29</v>
+      </c>
+      <c r="C40" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="D40" s="22">
+        <v>1</v>
+      </c>
+      <c r="E40" s="57">
+        <f>E39</f>
+        <v>45684</v>
+      </c>
+      <c r="F40" s="57">
+        <f>F39</f>
+        <v>45686</v>
+      </c>
+      <c r="G40" s="10">
+        <f>IF(OR(ISBLANK(inizio_attività),ISBLANK(fine_attività)),"",fine_attività-inizio_attività+1)</f>
+        <v>3</v>
+      </c>
+      <c r="H40" s="71"/>
+      <c r="I40" s="71"/>
+      <c r="J40" s="71"/>
+      <c r="K40" s="71"/>
+      <c r="L40" s="71"/>
+      <c r="M40" s="71"/>
+      <c r="N40" s="71"/>
+      <c r="O40" s="71"/>
+      <c r="P40" s="71"/>
+      <c r="Q40" s="71"/>
+      <c r="R40" s="64"/>
+      <c r="S40" s="23"/>
+      <c r="T40" s="64"/>
+      <c r="U40" s="64"/>
+      <c r="V40" s="64"/>
+      <c r="W40" s="64"/>
+      <c r="X40" s="64"/>
+      <c r="Y40" s="64"/>
+      <c r="Z40" s="23"/>
+      <c r="AA40" s="23"/>
+      <c r="AB40" s="23"/>
+      <c r="AC40" s="23"/>
+      <c r="AD40" s="23"/>
+      <c r="AE40" s="23"/>
+      <c r="AF40" s="23"/>
+      <c r="AG40" s="23"/>
+      <c r="AH40" s="23"/>
+      <c r="AI40" s="23"/>
+      <c r="AJ40" s="23"/>
+      <c r="AK40" s="23"/>
+      <c r="AL40" s="23"/>
+      <c r="AM40" s="23"/>
+      <c r="AN40" s="23"/>
+      <c r="AO40" s="23"/>
+      <c r="AP40" s="23"/>
+      <c r="AQ40" s="23"/>
+      <c r="AR40" s="23"/>
+      <c r="AS40" s="23"/>
+      <c r="AT40" s="23"/>
+      <c r="AU40" s="23"/>
+      <c r="AV40" s="23"/>
+      <c r="AW40" s="23"/>
+      <c r="AX40" s="23"/>
+      <c r="AY40" s="23"/>
+      <c r="AZ40" s="23"/>
+      <c r="BA40" s="23"/>
+      <c r="BB40" s="23"/>
+      <c r="BC40" s="23"/>
+      <c r="BD40" s="23"/>
+    </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="C3:D3"/>
@@ -4668,7 +4753,7 @@
     <mergeCell ref="V4:AB4"/>
     <mergeCell ref="AC4:AI4"/>
   </mergeCells>
-  <conditionalFormatting sqref="D7:D39">
+  <conditionalFormatting sqref="D7:D40">
     <cfRule type="dataBar" priority="17">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -4682,32 +4767,32 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:BC39">
+  <conditionalFormatting sqref="H5:BC40">
     <cfRule type="expression" dxfId="4" priority="3">
       <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:BC39">
+  <conditionalFormatting sqref="H7:BC40">
     <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
       <formula>AND(fine_attività&gt;=H$5,inizio_attività&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:BD39">
+  <conditionalFormatting sqref="H7:BD40">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>AND(inizio_attività&lt;=H$5,ROUNDDOWN((fine_attività-inizio_attività+1)*avanzamento_attività,0)+inizio_attività-1&gt;=H$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BD5:BD39">
+  <conditionalFormatting sqref="BD5:BD40">
     <cfRule type="expression" dxfId="1" priority="38">
       <formula>AND(TODAY()&gt;=BD$5,TODAY()&lt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BD7:BD39">
+  <conditionalFormatting sqref="BD7:BD40">
     <cfRule type="expression" dxfId="0" priority="42" stopIfTrue="1">
       <formula>AND(fine_attività&gt;=BD$5,inizio_attività&lt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" promptTitle="Visualizza settimana:" prompt="Cambiando questo numero si scorre la visualizzazione del diagramma di Gantt." sqref="E4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1</formula1>
     </dataValidation>
@@ -4734,7 +4819,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D7:D39</xm:sqref>
+          <xm:sqref>D7:D40</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4750,13 +4835,13 @@
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="62"/>
       <c r="B1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="63"/>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -4765,23 +4850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101003574973502B84C42B74035BA8AADE1A3" ma:contentTypeVersion="9" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="1ba771f4a91505810405fb99ac35d176">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8f4f0557-6568-4af7-94c6-f11cb446b9b2" xmlns:ns4="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3481e8909782aae8d117dfcc8e1ba87" ns3:_="" ns4:_="">
     <xsd:import namespace="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
@@ -4976,32 +5044,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A7A2A5-3EAC-4111-8CE5-4F4CD491981F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5018,4 +5078,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="8f4f0557-6568-4af7-94c6-f11cb446b9b2"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="5a27f7c0-5079-4b07-ba64-6dc03dd2d3af"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>